<commit_message>
feat(refactor): fix P0/P1/P2 audit issues, optimize tracker/db, add report generators and real-time metrics
</commit_message>
<xml_diff>
--- a/docs/PDR_Evaluation_Dashboard.xlsx
+++ b/docs/PDR_Evaluation_Dashboard.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>Thành phần</t>
   </si>
@@ -68,13 +68,16 @@
   </si>
   <si>
     <t>Real-time (25+ FPS)</t>
+  </si>
+  <si>
+    <t>⚠️ SỐ LIỆU DEMO — CHƯA ĐO THẬT ⚠️</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,6 +89,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -117,9 +128,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -144,7 +156,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Độ trễ xử lý theo từng module</a:t>
+              <a:t>Độ trễ xử lý theo từng module (cuda (NVIDIA GeForce GTX 1650))</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -192,19 +204,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>12.5</c:v>
+                  <c:v>11.71</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.1</c:v>
+                  <c:v>12.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.8</c:v>
+                  <c:v>0.45</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>11.2</c:v>
+                  <c:v>10.45</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>26.6</c:v>
+                  <c:v>12.29</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -592,13 +604,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="4" width="25.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -612,12 +624,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2">
-        <v>12.5</v>
+        <v>11.71</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
@@ -626,12 +638,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>7</v>
       </c>
       <c r="B3">
-        <v>2.1</v>
+        <v>12.2</v>
       </c>
       <c r="C3" t="s">
         <v>8</v>
@@ -640,12 +652,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>9</v>
       </c>
       <c r="B4">
-        <v>0.8</v>
+        <v>0.45</v>
       </c>
       <c r="C4" t="s">
         <v>10</v>
@@ -654,12 +666,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>12</v>
       </c>
       <c r="B5">
-        <v>11.2</v>
+        <v>10.45</v>
       </c>
       <c r="C5" t="s">
         <v>13</v>
@@ -668,12 +680,12 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>15</v>
       </c>
       <c r="B6">
-        <v>26.6</v>
+        <v>12.29</v>
       </c>
       <c r="C6" t="s">
         <v>16</v>
@@ -682,7 +694,19 @@
         <v>17</v>
       </c>
     </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A7:E7"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(P0-P2): remove hard-coded benchmark data, fix CSV watermark, prove pipeline CSV data, fix README description
</commit_message>
<xml_diff>
--- a/docs/PDR_Evaluation_Dashboard.xlsx
+++ b/docs/PDR_Evaluation_Dashboard.xlsx
@@ -7,77 +7,108 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="System Metrics" sheetId="1" r:id="rId1"/>
+    <sheet name="Benchmark" sheetId="1" r:id="rId1"/>
+    <sheet name="PAR Evaluation" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
-  <si>
-    <t>Thành phần</t>
-  </si>
-  <si>
-    <t>Độ trễ trung bình (ms)</t>
-  </si>
-  <si>
-    <t>Tối ưu hóa</t>
-  </si>
-  <si>
-    <t>Tốc độ khung hình kỳ vọng</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="29">
+  <si>
+    <t>HỆ THỐNG PDR — KẾT QUẢ BENCHMARK THỰC ĐO</t>
+  </si>
+  <si>
+    <t>Thiết bị: cuda (NVIDIA GeForce GTX 1650)</t>
+  </si>
+  <si>
+    <t>Thời điểm: 2026-09-08T20:29:29.294194</t>
+  </si>
+  <si>
+    <t>Module / Thuật toán</t>
+  </si>
+  <si>
+    <t>Độ trễ TB (ms)</t>
+  </si>
+  <si>
+    <t>Độ lệch chuẩn (ms)</t>
+  </si>
+  <si>
+    <t>FPS</t>
   </si>
   <si>
     <t>YOLOv8 Detection</t>
   </si>
   <si>
-    <t>TensorRT / Half Precision</t>
-  </si>
-  <si>
-    <t>30 FPS</t>
-  </si>
-  <si>
     <t>ByteTrack MOT</t>
   </si>
   <si>
-    <t>Matrix Operations</t>
-  </si>
-  <si>
     <t>K-Means Color HSV</t>
   </si>
   <si>
-    <t>Crop ROI xám hóa (Gray-world)</t>
-  </si>
-  <si>
-    <t>&gt; 60 FPS</t>
-  </si>
-  <si>
     <t>ResNet50 PAR</t>
   </si>
   <si>
-    <t>Batch Inference (2 crops/batch)</t>
-  </si>
-  <si>
-    <t>25 FPS</t>
+    <t>Attribute Matching Engine</t>
   </si>
   <si>
     <t>Overall Pipeline</t>
   </si>
   <si>
-    <t>Load Budgeting (Limit 2 CNN)</t>
-  </si>
-  <si>
-    <t>Real-time (25+ FPS)</t>
-  </si>
-  <si>
-    <t>⚠️ SỐ LIỆU DEMO — CHƯA ĐO THẬT ⚠️</t>
+    <t>HỆ THỐNG PDR — KẾT QUẢ ĐÁNH GIÁ MÔ HÌNH PAR</t>
+  </si>
+  <si>
+    <t>Thiết bị: Colab T4 GPU (Demo)</t>
+  </si>
+  <si>
+    <t>Mean Accuracy (mA): 89.33%</t>
+  </si>
+  <si>
+    <t>⚠️ SỐ LIỆU DEMO (Colab) — CHƯA ĐO THẬT TRÊN PA-100K ⚠️</t>
+  </si>
+  <si>
+    <t>Thuộc tính</t>
+  </si>
+  <si>
+    <t>Accuracy</t>
+  </si>
+  <si>
+    <t>Ghi chú</t>
+  </si>
+  <si>
+    <t>gender_female</t>
+  </si>
+  <si>
+    <t>85.20%</t>
+  </si>
+  <si>
+    <t>Cần dataset PA-100K để tính</t>
+  </si>
+  <si>
+    <t>hat</t>
+  </si>
+  <si>
+    <t>84.70%</t>
+  </si>
+  <si>
+    <t>glasses</t>
+  </si>
+  <si>
+    <t>91.00%</t>
+  </si>
+  <si>
+    <t>backpack</t>
+  </si>
+  <si>
+    <t>96.70%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -87,8 +118,24 @@
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <color rgb="FF1A2980"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -116,7 +163,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -124,14 +171,34 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -156,7 +223,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Độ trễ xử lý theo từng module (cuda (NVIDIA GeForce GTX 1650))</a:t>
+              <a:t>Độ trễ từng module — cuda (NVIDIA GeForce GTX 1650)</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -172,13 +239,18 @@
           <c:idx val="0"/>
           <c:order val="0"/>
           <c:tx>
-            <c:v>Độ trễ (ms)</c:v>
+            <c:v>Độ trễ trung bình (ms)</c:v>
           </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4F81BD"/>
+            </a:solidFill>
+          </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>'System Metrics'!$A$2:$A$6</c:f>
+              <c:f>Benchmark!$A$6:$A$11</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>YOLOv8 Detection</c:v>
                 </c:pt>
@@ -192,6 +264,9 @@
                   <c:v>ResNet50 PAR</c:v>
                 </c:pt>
                 <c:pt idx="4">
+                  <c:v>Attribute Matching Engine</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>Overall Pipeline</c:v>
                 </c:pt>
               </c:strCache>
@@ -199,24 +274,27 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'System Metrics'!$B$2:$B$6</c:f>
+              <c:f>Benchmark!$B$6:$B$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>11.71</c:v>
+                  <c:v>12.23</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12.2</c:v>
+                  <c:v>13.73</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.45</c:v>
+                  <c:v>0.55</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>10.45</c:v>
+                  <c:v>11.58</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>12.29</c:v>
+                  <c:v>0.0027</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>13.94</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -231,6 +309,24 @@
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Module</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50010002"/>
         <c:crosses val="autoZero"/>
@@ -290,14 +386,14 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>8</xdr:row>
+      <xdr:row>12</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>1143000</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1114425</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -604,110 +700,226 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="4" width="25.7109375" customWidth="1"/>
+    <col min="1" max="4" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
+      <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2">
-        <v>11.71</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D5" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
+    <row r="6" spans="1:4">
+      <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3">
-        <v>12.2</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B6" s="3">
+        <v>12.23</v>
+      </c>
+      <c r="C6" s="3">
+        <v>1.57</v>
+      </c>
+      <c r="D6" s="3">
+        <v>81.7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
+      <c r="B7" s="3">
+        <v>13.73</v>
+      </c>
+      <c r="C7" s="3">
+        <v>2.21</v>
+      </c>
+      <c r="D7" s="3">
+        <v>72.90000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B4">
-        <v>0.45</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B8" s="3">
+        <v>0.55</v>
+      </c>
+      <c r="C8" s="3">
+        <v>0.23</v>
+      </c>
+      <c r="D8" s="3">
+        <v>1821.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D4" t="s">
+      <c r="B9" s="3">
+        <v>11.58</v>
+      </c>
+      <c r="C9" s="3">
+        <v>1.23</v>
+      </c>
+      <c r="D9" s="3">
+        <v>86.3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
+      <c r="B10" s="3">
+        <v>0.0027</v>
+      </c>
+      <c r="C10" s="3">
+        <v>0.0001</v>
+      </c>
+      <c r="D10" s="3">
+        <v>367646.8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B5">
-        <v>10.45</v>
-      </c>
-      <c r="C5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6">
-        <v>12.29</v>
-      </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+      <c r="B11" s="3">
+        <v>13.94</v>
+      </c>
+      <c r="C11" s="3">
+        <v>1.86</v>
+      </c>
+      <c r="D11" s="3">
+        <v>71.7</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A7:E7"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="3" width="18.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A4:I4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>